<commit_message>
feat: System hardening - Risk tiers, Stale detection, Objective KPIs, Approval Escalation
</commit_message>
<xml_diff>
--- a/TurboFix-Tracker.xlsx
+++ b/TurboFix-Tracker.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Companies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Machines" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tickets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="MachineEvents" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Users" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Documents" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SpareParts" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Consumables" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Dashboard" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machines" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MachineEvents" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpareParts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumables" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,6 +512,11 @@
           <t>approved</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>payment_screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -539,6 +545,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -567,6 +574,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -584,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -595,7 +603,8 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col hidden="1" width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -641,6 +650,11 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>supervisor_id</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>has_open_tickets</t>
         </is>
       </c>
@@ -682,7 +696,12 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>U-ACME3-003</t>
+        </is>
+      </c>
+      <c r="J2">
         <f>COUNTIFS(Tickets!$B:$B,A2,Tickets!$J:$J,"Open")</f>
         <v/>
       </c>
@@ -724,7 +743,12 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>U-ACME3-003</t>
+        </is>
+      </c>
+      <c r="J3">
         <f>COUNTIFS(Tickets!$B:$B,A3,Tickets!$J:$J,"Open")</f>
         <v/>
       </c>
@@ -762,7 +786,8 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4">
         <f>COUNTIFS(Tickets!$B:$B,A4,Tickets!$J:$J,"Open")</f>
         <v/>
       </c>
@@ -800,7 +825,8 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5">
         <f>COUNTIFS(Tickets!$B:$B,A5,Tickets!$J:$J,"Open")</f>
         <v/>
       </c>
@@ -1424,7 +1450,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>$2b$12$cbdIgmMzyQK2CgvvpTIW0uzOSzm/XuWL/cr6yWXRqxSt6Tc0Q1ZNe</t>
+          <t>$2b$12$v0uajli.1Ze0em9AHlNb2eGj.ZGvBimjoMS3Rjrvt0cjrNCqgHIZa</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -1464,7 +1490,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>$2b$12$py3LEqaSvv/KbjFVolNYXuNb6OR4JfCJBW88GlDzSYANKIZQYlDmK</t>
+          <t>$2b$12$IIvHgLANrQHzvmovuC8DHeK1UOZ/NlBVCB8PU9JoFFlP7u7iTzxQ6</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -1504,7 +1530,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$2b$12$CMiMXfY41vAguGrm8RuqAO7RrkPCkvuwgc0S0jwm0fWBfu.k71Uoe</t>
+          <t>$2b$12$wTzN5JRTGMrvwdzyAK3fQenhV/J9scY7Ir9xwxd5v32TE3vwfvW6.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -1544,7 +1570,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>$2b$12$wLKghGUEvUf9WtumfFrnt.wF1CGUMOaDaGquKS7A01Q36b0dOUCNC</t>
+          <t>$2b$12$O3UGekcdmnN.XDFnSUY9VOCucahyrFJGXNj0KG9p3oV8T70XzXTaW</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -1584,7 +1610,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>$2b$12$BxMeMpvi1P1m6PtPf0kdoO0bqnB0FL.blFv8Upex9vcED.7ie4bE2</t>
+          <t>$2b$12$NOYeMQ4zcACgCXfmSC/0QOP3FOfgP51eH15cenT6fQuyXuqvO8DPq</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">

</xml_diff>